<commit_message>
feat: migrar aplicacion a Streamlit con diseno de circo digital e inteligencia artificial
</commit_message>
<xml_diff>
--- a/matriz_personalidades.xlsx
+++ b/matriz_personalidades.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ORACLE AI ONE\PROYECTO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ORACLE_AI_ONE\PROYECTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5637F518-3CE5-487D-BCF6-D38E56DC667E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73F8C742-BD52-4075-A711-344EF1EA5401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{68570187-7760-4693-9380-37FE8EE7F479}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="799" uniqueCount="594">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="799" uniqueCount="593">
   <si>
     <t>Harry Potter</t>
   </si>
@@ -189,9 +189,6 @@
     <t>Kenny McCormick</t>
   </si>
   <si>
-    <t>Jesse Pinkman (alt)</t>
-  </si>
-  <si>
     <t>ESTP</t>
   </si>
   <si>
@@ -213,9 +210,6 @@
     <t>Ron Weasley</t>
   </si>
   <si>
-    <t>Lindsay Bluth (alt)</t>
-  </si>
-  <si>
     <t>Randy Marsh</t>
   </si>
   <si>
@@ -228,9 +222,6 @@
     <t>Sirius Black</t>
   </si>
   <si>
-    <t>Gob Bluth (alt)</t>
-  </si>
-  <si>
     <t>Towelie</t>
   </si>
   <si>
@@ -246,21 +237,12 @@
     <t>Oscar Bluth</t>
   </si>
   <si>
-    <t>Eric Cartman (alt)</t>
-  </si>
-  <si>
-    <t>Saul Goodman (alt)</t>
-  </si>
-  <si>
     <t>ESTJ</t>
   </si>
   <si>
     <t>Minerva McGonagall</t>
   </si>
   <si>
-    <t>Lucille Bluth (alt)</t>
-  </si>
-  <si>
     <t>Clyde Donovan</t>
   </si>
   <si>
@@ -282,12 +264,6 @@
     <t>ENFJ</t>
   </si>
   <si>
-    <t>Albus Dumbledore (alt)</t>
-  </si>
-  <si>
-    <t>Michael Bluth (alt)</t>
-  </si>
-  <si>
     <t>Chef</t>
   </si>
   <si>
@@ -1828,6 +1804,27 @@
   </si>
   <si>
     <t>allows mobilizing resources at scale and optimizing architecture with implacable logic.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Michael Bluth </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lucille Bluth </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gob Bluth </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lindsay Bluth </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eric Cartman </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saul Goodman </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jesse Pinkman </t>
   </si>
 </sst>
 </file>
@@ -2224,145 +2221,145 @@
   <sheetData>
     <row r="1" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="B1" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="C1" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="D1" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="E1" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="F1" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="G1" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="H1" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="I1" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="J1" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="K1" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="L1" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="M1" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="N1" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
       <c r="O1" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="P1" t="s">
-        <v>273</v>
+        <v>265</v>
       </c>
       <c r="Q1" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="R1" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="S1" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="T1" t="s">
-        <v>299</v>
+        <v>291</v>
       </c>
       <c r="U1" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="V1" t="s">
+        <v>167</v>
+      </c>
+      <c r="W1" t="s">
+        <v>318</v>
+      </c>
+      <c r="X1" t="s">
+        <v>309</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>168</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>351</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>310</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>169</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>384</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>311</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>170</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>417</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>171</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>434</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>467</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>173</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>484</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>174</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>502</v>
+      </c>
+      <c r="AO1" t="s">
         <v>175</v>
       </c>
-      <c r="W1" t="s">
-        <v>326</v>
-      </c>
-      <c r="X1" t="s">
-        <v>317</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>176</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>359</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>318</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>177</v>
-      </c>
-      <c r="AC1" t="s">
-        <v>392</v>
-      </c>
-      <c r="AD1" t="s">
-        <v>319</v>
-      </c>
-      <c r="AE1" t="s">
-        <v>178</v>
-      </c>
-      <c r="AF1" t="s">
-        <v>425</v>
-      </c>
-      <c r="AG1" t="s">
-        <v>179</v>
-      </c>
-      <c r="AH1" t="s">
-        <v>442</v>
-      </c>
-      <c r="AI1" t="s">
-        <v>180</v>
-      </c>
-      <c r="AJ1" t="s">
-        <v>475</v>
-      </c>
-      <c r="AK1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AL1" t="s">
-        <v>492</v>
-      </c>
-      <c r="AM1" t="s">
-        <v>182</v>
-      </c>
-      <c r="AN1" t="s">
-        <v>510</v>
-      </c>
-      <c r="AO1" t="s">
-        <v>183</v>
-      </c>
       <c r="AP1" t="s">
-        <v>526</v>
+        <v>518</v>
       </c>
       <c r="AQ1" t="s">
-        <v>543</v>
+        <v>535</v>
       </c>
       <c r="AR1" t="s">
-        <v>543</v>
+        <v>535</v>
       </c>
       <c r="AS1" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="AT1" t="s">
-        <v>560</v>
+        <v>552</v>
       </c>
       <c r="AU1" t="s">
-        <v>577</v>
+        <v>569</v>
       </c>
     </row>
     <row r="2" spans="1:47" x14ac:dyDescent="0.25">
@@ -2373,139 +2370,139 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="D2" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="E2" t="s">
         <v>44</v>
       </c>
       <c r="F2" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="G2" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="H2" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="I2" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="J2" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="K2" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="L2" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="M2" t="s">
         <v>2</v>
       </c>
       <c r="N2" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="O2" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="P2" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
       <c r="Q2" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="R2" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="S2" t="s">
-        <v>283</v>
+        <v>275</v>
       </c>
       <c r="T2" t="s">
-        <v>300</v>
+        <v>292</v>
       </c>
       <c r="U2" t="s">
         <v>3</v>
       </c>
       <c r="V2" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="W2" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
       <c r="X2" t="s">
         <v>4</v>
       </c>
       <c r="Y2" t="s">
-        <v>343</v>
+        <v>335</v>
       </c>
       <c r="Z2" t="s">
-        <v>360</v>
+        <v>352</v>
       </c>
       <c r="AA2" t="s">
         <v>5</v>
       </c>
       <c r="AB2" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="AC2" t="s">
-        <v>393</v>
+        <v>385</v>
       </c>
       <c r="AD2" t="s">
         <v>6</v>
       </c>
       <c r="AE2" t="s">
-        <v>409</v>
+        <v>401</v>
       </c>
       <c r="AF2" t="s">
-        <v>426</v>
+        <v>418</v>
       </c>
       <c r="AG2" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="AH2" t="s">
-        <v>443</v>
+        <v>435</v>
       </c>
       <c r="AI2" t="s">
-        <v>459</v>
+        <v>451</v>
       </c>
       <c r="AJ2" t="s">
-        <v>476</v>
+        <v>468</v>
       </c>
       <c r="AK2" t="s">
-        <v>509</v>
+        <v>501</v>
       </c>
       <c r="AL2" t="s">
-        <v>493</v>
+        <v>485</v>
       </c>
       <c r="AM2" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="AN2" t="s">
-        <v>493</v>
+        <v>485</v>
       </c>
       <c r="AO2" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="AP2" t="s">
-        <v>527</v>
+        <v>519</v>
       </c>
       <c r="AQ2" t="s">
-        <v>544</v>
+        <v>536</v>
       </c>
       <c r="AR2" t="s">
-        <v>544</v>
+        <v>536</v>
       </c>
       <c r="AS2" t="s">
         <v>7</v>
       </c>
       <c r="AT2" t="s">
-        <v>561</v>
+        <v>553</v>
       </c>
       <c r="AU2" t="s">
-        <v>578</v>
+        <v>570</v>
       </c>
     </row>
     <row r="3" spans="1:47" x14ac:dyDescent="0.25">
@@ -2516,139 +2513,139 @@
         <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="D3" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="E3" t="s">
         <v>44</v>
       </c>
       <c r="F3" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="G3" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="H3" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="I3" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="J3" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="K3" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="L3" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="M3" t="s">
         <v>9</v>
       </c>
       <c r="N3" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="O3" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="P3" t="s">
-        <v>275</v>
+        <v>267</v>
       </c>
       <c r="Q3" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="R3" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="S3" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="T3" t="s">
-        <v>301</v>
+        <v>293</v>
       </c>
       <c r="U3" t="s">
         <v>10</v>
       </c>
       <c r="V3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="W3" t="s">
-        <v>328</v>
+        <v>320</v>
       </c>
       <c r="X3" t="s">
         <v>11</v>
       </c>
       <c r="Y3" t="s">
-        <v>344</v>
+        <v>336</v>
       </c>
       <c r="Z3" t="s">
-        <v>361</v>
+        <v>353</v>
       </c>
       <c r="AA3" t="s">
         <v>12</v>
       </c>
       <c r="AB3" t="s">
-        <v>377</v>
+        <v>369</v>
       </c>
       <c r="AC3" t="s">
-        <v>394</v>
+        <v>386</v>
       </c>
       <c r="AD3" t="s">
         <v>13</v>
       </c>
       <c r="AE3" t="s">
-        <v>410</v>
+        <v>402</v>
       </c>
       <c r="AF3" t="s">
-        <v>427</v>
+        <v>419</v>
       </c>
       <c r="AG3" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AH3" t="s">
-        <v>444</v>
+        <v>436</v>
       </c>
       <c r="AI3" t="s">
-        <v>460</v>
+        <v>452</v>
       </c>
       <c r="AJ3" t="s">
-        <v>477</v>
+        <v>469</v>
       </c>
       <c r="AK3" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="AL3" t="s">
-        <v>494</v>
+        <v>486</v>
       </c>
       <c r="AM3" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="AN3" t="s">
-        <v>511</v>
+        <v>503</v>
       </c>
       <c r="AO3" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="AP3" t="s">
-        <v>528</v>
+        <v>520</v>
       </c>
       <c r="AQ3" t="s">
-        <v>545</v>
+        <v>537</v>
       </c>
       <c r="AR3" t="s">
-        <v>545</v>
+        <v>537</v>
       </c>
       <c r="AS3" t="s">
         <v>14</v>
       </c>
       <c r="AT3" t="s">
-        <v>562</v>
+        <v>554</v>
       </c>
       <c r="AU3" t="s">
-        <v>579</v>
+        <v>571</v>
       </c>
     </row>
     <row r="4" spans="1:47" x14ac:dyDescent="0.25">
@@ -2659,139 +2656,139 @@
         <v>15</v>
       </c>
       <c r="C4" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="D4" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="E4" t="s">
         <v>9</v>
       </c>
       <c r="F4" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="G4" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="H4" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="I4" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="J4" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="K4" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="L4" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="M4" t="s">
         <v>16</v>
       </c>
       <c r="N4" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="O4" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="P4" t="s">
-        <v>276</v>
+        <v>268</v>
       </c>
       <c r="Q4" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="R4" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="S4" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="T4" t="s">
-        <v>302</v>
+        <v>294</v>
       </c>
       <c r="U4" t="s">
         <v>17</v>
       </c>
       <c r="V4" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="W4" t="s">
-        <v>329</v>
+        <v>321</v>
       </c>
       <c r="X4" t="s">
         <v>18</v>
       </c>
       <c r="Y4" t="s">
-        <v>345</v>
+        <v>337</v>
       </c>
       <c r="Z4" t="s">
-        <v>362</v>
+        <v>354</v>
       </c>
       <c r="AA4" t="s">
         <v>19</v>
       </c>
       <c r="AB4" t="s">
-        <v>378</v>
+        <v>370</v>
       </c>
       <c r="AC4" t="s">
-        <v>395</v>
+        <v>387</v>
       </c>
       <c r="AD4" t="s">
         <v>20</v>
       </c>
       <c r="AE4" t="s">
-        <v>411</v>
+        <v>403</v>
       </c>
       <c r="AF4" t="s">
-        <v>428</v>
+        <v>420</v>
       </c>
       <c r="AG4" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="AH4" t="s">
-        <v>445</v>
+        <v>437</v>
       </c>
       <c r="AI4" t="s">
-        <v>461</v>
+        <v>453</v>
       </c>
       <c r="AJ4" t="s">
-        <v>478</v>
+        <v>470</v>
       </c>
       <c r="AK4" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="AL4" t="s">
-        <v>495</v>
+        <v>487</v>
       </c>
       <c r="AM4" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="AN4" t="s">
-        <v>512</v>
+        <v>504</v>
       </c>
       <c r="AO4" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="AP4" t="s">
-        <v>529</v>
+        <v>521</v>
       </c>
       <c r="AQ4" t="s">
-        <v>546</v>
+        <v>538</v>
       </c>
       <c r="AR4" t="s">
-        <v>546</v>
+        <v>538</v>
       </c>
       <c r="AS4" t="s">
         <v>21</v>
       </c>
       <c r="AT4" t="s">
-        <v>563</v>
+        <v>555</v>
       </c>
       <c r="AU4" t="s">
-        <v>580</v>
+        <v>572</v>
       </c>
     </row>
     <row r="5" spans="1:47" x14ac:dyDescent="0.25">
@@ -2802,282 +2799,282 @@
         <v>22</v>
       </c>
       <c r="C5" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="D5" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="E5" t="s">
         <v>2</v>
       </c>
       <c r="F5" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="G5" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="H5" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="I5" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="J5" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="K5" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
       <c r="L5" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
       <c r="M5" t="s">
         <v>16</v>
       </c>
       <c r="N5" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="O5" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="P5" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="Q5" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="R5" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="S5" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="T5" t="s">
-        <v>303</v>
+        <v>295</v>
       </c>
       <c r="U5" t="s">
         <v>23</v>
       </c>
       <c r="V5" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="W5" t="s">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="X5" t="s">
         <v>24</v>
       </c>
       <c r="Y5" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="Z5" t="s">
-        <v>363</v>
+        <v>355</v>
       </c>
       <c r="AA5" t="s">
         <v>25</v>
       </c>
       <c r="AB5" t="s">
-        <v>379</v>
+        <v>371</v>
       </c>
       <c r="AC5" t="s">
-        <v>396</v>
+        <v>388</v>
       </c>
       <c r="AD5" t="s">
         <v>26</v>
       </c>
       <c r="AE5" t="s">
-        <v>412</v>
+        <v>404</v>
       </c>
       <c r="AF5" t="s">
-        <v>429</v>
+        <v>421</v>
       </c>
       <c r="AG5" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="AH5" t="s">
-        <v>446</v>
+        <v>438</v>
       </c>
       <c r="AI5" t="s">
-        <v>462</v>
+        <v>454</v>
       </c>
       <c r="AJ5" t="s">
-        <v>479</v>
+        <v>471</v>
       </c>
       <c r="AK5" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="AL5" t="s">
-        <v>496</v>
+        <v>488</v>
       </c>
       <c r="AM5" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="AN5" t="s">
-        <v>513</v>
+        <v>505</v>
       </c>
       <c r="AO5" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="AP5" t="s">
-        <v>530</v>
+        <v>522</v>
       </c>
       <c r="AQ5" t="s">
-        <v>547</v>
+        <v>539</v>
       </c>
       <c r="AR5" t="s">
-        <v>547</v>
+        <v>539</v>
       </c>
       <c r="AS5" t="s">
         <v>27</v>
       </c>
       <c r="AT5" t="s">
-        <v>564</v>
+        <v>556</v>
       </c>
       <c r="AU5" t="s">
-        <v>581</v>
+        <v>573</v>
       </c>
     </row>
     <row r="6" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="B6" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C6" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="D6" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="E6" t="s">
         <v>2</v>
       </c>
       <c r="F6" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="G6" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="H6" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="I6" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="J6" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="K6" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
       <c r="L6" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
       <c r="M6" t="s">
         <v>44</v>
       </c>
       <c r="N6" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="O6" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="P6" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="Q6" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="R6" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="S6" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
       <c r="T6" t="s">
-        <v>304</v>
+        <v>296</v>
       </c>
       <c r="U6" t="s">
         <v>28</v>
       </c>
       <c r="V6" t="s">
-        <v>324</v>
+        <v>316</v>
       </c>
       <c r="W6" t="s">
-        <v>331</v>
+        <v>323</v>
       </c>
       <c r="X6" t="s">
         <v>29</v>
       </c>
       <c r="Y6" t="s">
-        <v>347</v>
+        <v>339</v>
       </c>
       <c r="Z6" t="s">
-        <v>364</v>
+        <v>356</v>
       </c>
       <c r="AA6" t="s">
         <v>30</v>
       </c>
       <c r="AB6" t="s">
-        <v>380</v>
+        <v>372</v>
       </c>
       <c r="AC6" t="s">
-        <v>397</v>
+        <v>389</v>
       </c>
       <c r="AD6" t="s">
         <v>31</v>
       </c>
       <c r="AE6" t="s">
-        <v>413</v>
+        <v>405</v>
       </c>
       <c r="AF6" t="s">
-        <v>430</v>
+        <v>422</v>
       </c>
       <c r="AG6" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="AH6" t="s">
-        <v>447</v>
+        <v>439</v>
       </c>
       <c r="AI6" t="s">
-        <v>463</v>
+        <v>455</v>
       </c>
       <c r="AJ6" t="s">
-        <v>480</v>
+        <v>472</v>
       </c>
       <c r="AK6" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="AL6" t="s">
-        <v>497</v>
+        <v>489</v>
       </c>
       <c r="AM6" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="AN6" t="s">
-        <v>514</v>
+        <v>506</v>
       </c>
       <c r="AO6" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="AP6" t="s">
-        <v>531</v>
+        <v>523</v>
       </c>
       <c r="AQ6" t="s">
-        <v>548</v>
+        <v>540</v>
       </c>
       <c r="AR6" t="s">
-        <v>548</v>
+        <v>540</v>
       </c>
       <c r="AS6" t="s">
         <v>21</v>
       </c>
       <c r="AT6" t="s">
-        <v>565</v>
+        <v>557</v>
       </c>
       <c r="AU6" t="s">
-        <v>582</v>
+        <v>574</v>
       </c>
     </row>
     <row r="7" spans="1:47" x14ac:dyDescent="0.25">
@@ -3088,139 +3085,139 @@
         <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="D7" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="E7" t="s">
         <v>16</v>
       </c>
       <c r="F7" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="G7" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="H7" t="s">
+        <v>239</v>
+      </c>
+      <c r="I7" t="s">
+        <v>85</v>
+      </c>
+      <c r="J7" t="s">
+        <v>231</v>
+      </c>
+      <c r="K7" t="s">
         <v>247</v>
       </c>
-      <c r="I7" t="s">
-        <v>93</v>
-      </c>
-      <c r="J7" t="s">
-        <v>239</v>
-      </c>
-      <c r="K7" t="s">
-        <v>255</v>
-      </c>
       <c r="L7" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="M7" t="s">
         <v>2</v>
       </c>
       <c r="N7" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="O7" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="P7" t="s">
-        <v>275</v>
+        <v>267</v>
       </c>
       <c r="Q7" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="R7" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="S7" t="s">
-        <v>288</v>
+        <v>280</v>
       </c>
       <c r="T7" t="s">
-        <v>305</v>
+        <v>297</v>
       </c>
       <c r="U7" t="s">
         <v>33</v>
       </c>
       <c r="V7" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="W7" t="s">
-        <v>332</v>
+        <v>324</v>
       </c>
       <c r="X7" t="s">
         <v>34</v>
       </c>
       <c r="Y7" t="s">
-        <v>348</v>
+        <v>340</v>
       </c>
       <c r="Z7" t="s">
-        <v>365</v>
+        <v>357</v>
       </c>
       <c r="AA7" t="s">
         <v>35</v>
       </c>
       <c r="AB7" t="s">
-        <v>381</v>
+        <v>373</v>
       </c>
       <c r="AC7" t="s">
-        <v>398</v>
+        <v>390</v>
       </c>
       <c r="AD7" t="s">
         <v>36</v>
       </c>
       <c r="AE7" t="s">
-        <v>414</v>
+        <v>406</v>
       </c>
       <c r="AF7" t="s">
-        <v>431</v>
+        <v>423</v>
       </c>
       <c r="AG7" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="AH7" t="s">
-        <v>448</v>
+        <v>440</v>
       </c>
       <c r="AI7" t="s">
-        <v>464</v>
+        <v>456</v>
       </c>
       <c r="AJ7" t="s">
-        <v>481</v>
+        <v>473</v>
       </c>
       <c r="AK7" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="AL7" t="s">
-        <v>498</v>
+        <v>490</v>
       </c>
       <c r="AM7" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="AN7" t="s">
-        <v>515</v>
+        <v>507</v>
       </c>
       <c r="AO7" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="AP7" t="s">
-        <v>532</v>
+        <v>524</v>
       </c>
       <c r="AQ7" t="s">
-        <v>549</v>
+        <v>541</v>
       </c>
       <c r="AR7" t="s">
-        <v>549</v>
+        <v>541</v>
       </c>
       <c r="AS7" t="s">
         <v>37</v>
       </c>
       <c r="AT7" t="s">
-        <v>566</v>
+        <v>558</v>
       </c>
       <c r="AU7" t="s">
-        <v>583</v>
+        <v>575</v>
       </c>
     </row>
     <row r="8" spans="1:47" x14ac:dyDescent="0.25">
@@ -3231,139 +3228,139 @@
         <v>38</v>
       </c>
       <c r="C8" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="D8" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="E8" t="s">
         <v>16</v>
       </c>
       <c r="F8" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="G8" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="H8" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="I8" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="J8" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="K8" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="L8" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="M8" t="s">
         <v>9</v>
       </c>
       <c r="N8" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="O8" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="P8" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
       <c r="Q8" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="R8" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="S8" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="T8" t="s">
-        <v>306</v>
+        <v>298</v>
       </c>
       <c r="U8" t="s">
         <v>39</v>
       </c>
       <c r="V8" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="W8" t="s">
-        <v>333</v>
+        <v>325</v>
       </c>
       <c r="X8" t="s">
         <v>40</v>
       </c>
       <c r="Y8" t="s">
-        <v>349</v>
+        <v>341</v>
       </c>
       <c r="Z8" t="s">
-        <v>366</v>
+        <v>358</v>
       </c>
       <c r="AA8" t="s">
         <v>41</v>
       </c>
       <c r="AB8" t="s">
-        <v>382</v>
+        <v>374</v>
       </c>
       <c r="AC8" t="s">
-        <v>399</v>
+        <v>391</v>
       </c>
       <c r="AD8" t="s">
         <v>42</v>
       </c>
       <c r="AE8" t="s">
-        <v>415</v>
+        <v>407</v>
       </c>
       <c r="AF8" t="s">
-        <v>432</v>
+        <v>424</v>
       </c>
       <c r="AG8" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="AH8" t="s">
-        <v>449</v>
+        <v>441</v>
       </c>
       <c r="AI8" t="s">
-        <v>465</v>
+        <v>457</v>
       </c>
       <c r="AJ8" t="s">
-        <v>482</v>
+        <v>474</v>
       </c>
       <c r="AK8" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="AL8" t="s">
-        <v>499</v>
+        <v>491</v>
       </c>
       <c r="AM8" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="AN8" t="s">
-        <v>516</v>
+        <v>508</v>
       </c>
       <c r="AO8" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="AP8" t="s">
-        <v>533</v>
+        <v>525</v>
       </c>
       <c r="AQ8" t="s">
-        <v>550</v>
+        <v>542</v>
       </c>
       <c r="AR8" t="s">
-        <v>550</v>
+        <v>542</v>
       </c>
       <c r="AS8" t="s">
         <v>37</v>
       </c>
       <c r="AT8" t="s">
-        <v>567</v>
+        <v>559</v>
       </c>
       <c r="AU8" t="s">
-        <v>584</v>
+        <v>576</v>
       </c>
     </row>
     <row r="9" spans="1:47" x14ac:dyDescent="0.25">
@@ -3374,1283 +3371,1283 @@
         <v>43</v>
       </c>
       <c r="C9" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="D9" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="E9" t="s">
         <v>9</v>
       </c>
       <c r="F9" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="G9" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="H9" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="I9" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="J9" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="K9" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="L9" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
       <c r="M9" t="s">
         <v>44</v>
       </c>
       <c r="N9" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="O9" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="P9" t="s">
-        <v>276</v>
+        <v>268</v>
       </c>
       <c r="Q9" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="R9" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="S9" t="s">
-        <v>290</v>
+        <v>282</v>
       </c>
       <c r="T9" t="s">
-        <v>307</v>
+        <v>299</v>
       </c>
       <c r="U9" t="s">
         <v>0</v>
       </c>
       <c r="V9" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="W9" t="s">
-        <v>334</v>
+        <v>326</v>
       </c>
       <c r="X9" t="s">
         <v>45</v>
       </c>
       <c r="Y9" t="s">
-        <v>350</v>
+        <v>342</v>
       </c>
       <c r="Z9" t="s">
-        <v>367</v>
+        <v>359</v>
       </c>
       <c r="AA9" t="s">
         <v>46</v>
       </c>
       <c r="AB9" t="s">
-        <v>383</v>
+        <v>375</v>
       </c>
       <c r="AC9" t="s">
-        <v>400</v>
+        <v>392</v>
       </c>
       <c r="AD9" t="s">
-        <v>47</v>
+        <v>592</v>
       </c>
       <c r="AE9" t="s">
-        <v>416</v>
+        <v>408</v>
       </c>
       <c r="AF9" t="s">
-        <v>433</v>
+        <v>425</v>
       </c>
       <c r="AG9" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="AH9" t="s">
-        <v>450</v>
+        <v>442</v>
       </c>
       <c r="AI9" t="s">
-        <v>466</v>
+        <v>458</v>
       </c>
       <c r="AJ9" t="s">
-        <v>483</v>
+        <v>475</v>
       </c>
       <c r="AK9" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="AL9" t="s">
-        <v>500</v>
+        <v>492</v>
       </c>
       <c r="AM9" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="AN9" t="s">
-        <v>517</v>
+        <v>509</v>
       </c>
       <c r="AO9" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="AP9" t="s">
-        <v>534</v>
+        <v>526</v>
       </c>
       <c r="AQ9" t="s">
-        <v>551</v>
+        <v>543</v>
       </c>
       <c r="AR9" t="s">
-        <v>551</v>
+        <v>543</v>
       </c>
       <c r="AS9" t="s">
         <v>21</v>
       </c>
       <c r="AT9" t="s">
-        <v>568</v>
+        <v>560</v>
       </c>
       <c r="AU9" t="s">
-        <v>585</v>
+        <v>577</v>
       </c>
     </row>
     <row r="10" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C10" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="D10" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="E10" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="F10" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="G10" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="H10" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="I10" t="s">
         <v>2</v>
       </c>
       <c r="J10" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="K10" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="L10" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="M10" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="N10" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="O10" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="P10" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
       <c r="Q10" t="s">
         <v>44</v>
       </c>
       <c r="R10" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="S10" t="s">
-        <v>291</v>
+        <v>283</v>
       </c>
       <c r="T10" t="s">
-        <v>308</v>
+        <v>300</v>
       </c>
       <c r="U10" t="s">
+        <v>48</v>
+      </c>
+      <c r="V10" t="s">
+        <v>312</v>
+      </c>
+      <c r="W10" t="s">
+        <v>327</v>
+      </c>
+      <c r="X10" t="s">
         <v>49</v>
       </c>
-      <c r="V10" t="s">
-        <v>320</v>
-      </c>
-      <c r="W10" t="s">
-        <v>335</v>
-      </c>
-      <c r="X10" t="s">
+      <c r="Y10" t="s">
+        <v>343</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>360</v>
+      </c>
+      <c r="AA10" t="s">
         <v>50</v>
       </c>
-      <c r="Y10" t="s">
-        <v>351</v>
-      </c>
-      <c r="Z10" t="s">
-        <v>368</v>
-      </c>
-      <c r="AA10" t="s">
+      <c r="AB10" t="s">
+        <v>376</v>
+      </c>
+      <c r="AC10" t="s">
+        <v>393</v>
+      </c>
+      <c r="AD10" t="s">
         <v>51</v>
       </c>
-      <c r="AB10" t="s">
-        <v>384</v>
-      </c>
-      <c r="AC10" t="s">
-        <v>401</v>
-      </c>
-      <c r="AD10" t="s">
-        <v>52</v>
-      </c>
       <c r="AE10" t="s">
-        <v>417</v>
+        <v>409</v>
       </c>
       <c r="AF10" t="s">
-        <v>434</v>
+        <v>426</v>
       </c>
       <c r="AG10" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="AH10" t="s">
-        <v>451</v>
+        <v>443</v>
       </c>
       <c r="AI10" t="s">
-        <v>467</v>
+        <v>459</v>
       </c>
       <c r="AJ10" t="s">
-        <v>484</v>
+        <v>476</v>
       </c>
       <c r="AK10" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="AL10" t="s">
-        <v>501</v>
+        <v>493</v>
       </c>
       <c r="AM10" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="AN10" t="s">
-        <v>518</v>
+        <v>510</v>
       </c>
       <c r="AO10" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="AP10" t="s">
-        <v>535</v>
+        <v>527</v>
       </c>
       <c r="AQ10" t="s">
-        <v>552</v>
+        <v>544</v>
       </c>
       <c r="AR10" t="s">
-        <v>552</v>
+        <v>544</v>
       </c>
       <c r="AS10" t="s">
         <v>7</v>
       </c>
       <c r="AT10" t="s">
-        <v>569</v>
+        <v>561</v>
       </c>
       <c r="AU10" t="s">
-        <v>586</v>
+        <v>578</v>
       </c>
     </row>
     <row r="11" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C11" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="D11" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="E11" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="F11" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="G11" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="H11" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="I11" t="s">
         <v>9</v>
       </c>
       <c r="J11" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="K11" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="L11" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="M11" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="N11" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="O11" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="P11" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
       <c r="Q11" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="R11" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="S11" t="s">
-        <v>292</v>
+        <v>284</v>
       </c>
       <c r="T11" t="s">
-        <v>309</v>
+        <v>301</v>
       </c>
       <c r="U11" t="s">
+        <v>53</v>
+      </c>
+      <c r="V11" t="s">
+        <v>163</v>
+      </c>
+      <c r="W11" t="s">
+        <v>328</v>
+      </c>
+      <c r="X11" t="s">
+        <v>589</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>344</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>361</v>
+      </c>
+      <c r="AA11" t="s">
         <v>54</v>
       </c>
-      <c r="V11" t="s">
-        <v>171</v>
-      </c>
-      <c r="W11" t="s">
-        <v>336</v>
-      </c>
-      <c r="X11" t="s">
+      <c r="AB11" t="s">
+        <v>377</v>
+      </c>
+      <c r="AC11" t="s">
+        <v>394</v>
+      </c>
+      <c r="AD11" t="s">
         <v>55</v>
       </c>
-      <c r="Y11" t="s">
-        <v>352</v>
-      </c>
-      <c r="Z11" t="s">
-        <v>369</v>
-      </c>
-      <c r="AA11" t="s">
-        <v>56</v>
-      </c>
-      <c r="AB11" t="s">
-        <v>385</v>
-      </c>
-      <c r="AC11" t="s">
-        <v>402</v>
-      </c>
-      <c r="AD11" t="s">
-        <v>57</v>
-      </c>
       <c r="AE11" t="s">
-        <v>418</v>
+        <v>410</v>
       </c>
       <c r="AF11" t="s">
-        <v>435</v>
+        <v>427</v>
       </c>
       <c r="AG11" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="AH11" t="s">
-        <v>452</v>
+        <v>444</v>
       </c>
       <c r="AI11" t="s">
-        <v>468</v>
+        <v>460</v>
       </c>
       <c r="AJ11" t="s">
-        <v>485</v>
+        <v>477</v>
       </c>
       <c r="AK11" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="AL11" t="s">
-        <v>502</v>
+        <v>494</v>
       </c>
       <c r="AM11" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="AN11" t="s">
-        <v>519</v>
+        <v>511</v>
       </c>
       <c r="AO11" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="AP11" t="s">
-        <v>536</v>
+        <v>528</v>
       </c>
       <c r="AQ11" t="s">
-        <v>553</v>
+        <v>545</v>
       </c>
       <c r="AR11" t="s">
-        <v>553</v>
+        <v>545</v>
       </c>
       <c r="AS11" t="s">
         <v>21</v>
       </c>
       <c r="AT11" t="s">
-        <v>570</v>
+        <v>562</v>
       </c>
       <c r="AU11" t="s">
-        <v>587</v>
+        <v>579</v>
       </c>
     </row>
     <row r="12" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B12" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C12" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="D12" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="E12" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="F12" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="G12" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="H12" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="I12" t="s">
         <v>9</v>
       </c>
       <c r="J12" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="K12" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="L12" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="M12" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="N12" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="O12" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="P12" t="s">
-        <v>279</v>
+        <v>271</v>
       </c>
       <c r="Q12" t="s">
         <v>16</v>
       </c>
       <c r="R12" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="S12" t="s">
-        <v>293</v>
+        <v>285</v>
       </c>
       <c r="T12" t="s">
-        <v>310</v>
+        <v>302</v>
       </c>
       <c r="U12" t="s">
+        <v>57</v>
+      </c>
+      <c r="V12" t="s">
+        <v>164</v>
+      </c>
+      <c r="W12" t="s">
+        <v>329</v>
+      </c>
+      <c r="X12" t="s">
+        <v>588</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>345</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>362</v>
+      </c>
+      <c r="AA12" t="s">
+        <v>58</v>
+      </c>
+      <c r="AB12" t="s">
+        <v>378</v>
+      </c>
+      <c r="AC12" t="s">
+        <v>395</v>
+      </c>
+      <c r="AD12" t="s">
         <v>59</v>
       </c>
-      <c r="V12" t="s">
-        <v>172</v>
-      </c>
-      <c r="W12" t="s">
-        <v>337</v>
-      </c>
-      <c r="X12" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y12" t="s">
-        <v>353</v>
-      </c>
-      <c r="Z12" t="s">
-        <v>370</v>
-      </c>
-      <c r="AA12" t="s">
-        <v>61</v>
-      </c>
-      <c r="AB12" t="s">
-        <v>386</v>
-      </c>
-      <c r="AC12" t="s">
-        <v>403</v>
-      </c>
-      <c r="AD12" t="s">
-        <v>62</v>
-      </c>
       <c r="AE12" t="s">
-        <v>419</v>
+        <v>411</v>
       </c>
       <c r="AF12" t="s">
-        <v>436</v>
+        <v>428</v>
       </c>
       <c r="AG12" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="AH12" t="s">
-        <v>453</v>
+        <v>445</v>
       </c>
       <c r="AI12" t="s">
-        <v>469</v>
+        <v>461</v>
       </c>
       <c r="AJ12" t="s">
-        <v>486</v>
+        <v>478</v>
       </c>
       <c r="AK12" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="AL12" t="s">
-        <v>503</v>
+        <v>495</v>
       </c>
       <c r="AM12" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="AN12" t="s">
-        <v>520</v>
+        <v>512</v>
       </c>
       <c r="AO12" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="AP12" t="s">
-        <v>537</v>
+        <v>529</v>
       </c>
       <c r="AQ12" t="s">
-        <v>554</v>
+        <v>546</v>
       </c>
       <c r="AR12" t="s">
-        <v>554</v>
+        <v>546</v>
       </c>
       <c r="AS12" t="s">
         <v>7</v>
       </c>
       <c r="AT12" t="s">
-        <v>571</v>
+        <v>563</v>
       </c>
       <c r="AU12" t="s">
-        <v>588</v>
+        <v>580</v>
       </c>
     </row>
     <row r="13" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B13" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C13" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="D13" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="E13" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="F13" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="G13" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="H13" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="I13" t="s">
         <v>2</v>
       </c>
       <c r="J13" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="K13" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="L13" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="M13" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="N13" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="O13" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="P13" t="s">
-        <v>279</v>
+        <v>271</v>
       </c>
       <c r="Q13" t="s">
         <v>16</v>
       </c>
       <c r="R13" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="S13" t="s">
-        <v>294</v>
+        <v>286</v>
       </c>
       <c r="T13" t="s">
-        <v>311</v>
+        <v>303</v>
       </c>
       <c r="U13" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="V13" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="W13" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
       <c r="X13" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="Y13" t="s">
-        <v>354</v>
+        <v>346</v>
       </c>
       <c r="Z13" t="s">
-        <v>371</v>
+        <v>363</v>
       </c>
       <c r="AA13" t="s">
-        <v>66</v>
+        <v>590</v>
       </c>
       <c r="AB13" t="s">
-        <v>387</v>
+        <v>379</v>
       </c>
       <c r="AC13" t="s">
-        <v>404</v>
+        <v>396</v>
       </c>
       <c r="AD13" t="s">
-        <v>67</v>
+        <v>591</v>
       </c>
       <c r="AE13" t="s">
-        <v>420</v>
+        <v>412</v>
       </c>
       <c r="AF13" t="s">
-        <v>437</v>
+        <v>429</v>
       </c>
       <c r="AG13" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="AH13" t="s">
-        <v>454</v>
+        <v>446</v>
       </c>
       <c r="AI13" t="s">
-        <v>470</v>
+        <v>462</v>
       </c>
       <c r="AJ13" t="s">
-        <v>487</v>
+        <v>479</v>
       </c>
       <c r="AK13" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="AL13" t="s">
-        <v>504</v>
+        <v>496</v>
       </c>
       <c r="AM13" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="AN13" t="s">
-        <v>521</v>
+        <v>513</v>
       </c>
       <c r="AO13" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="AP13" t="s">
-        <v>538</v>
+        <v>530</v>
       </c>
       <c r="AQ13" t="s">
-        <v>555</v>
+        <v>547</v>
       </c>
       <c r="AR13" t="s">
-        <v>555</v>
+        <v>547</v>
       </c>
       <c r="AS13" t="s">
         <v>27</v>
       </c>
       <c r="AT13" t="s">
-        <v>572</v>
+        <v>564</v>
       </c>
       <c r="AU13" t="s">
-        <v>589</v>
+        <v>581</v>
       </c>
     </row>
     <row r="14" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="B14" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C14" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="D14" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="E14" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="F14" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="G14" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="H14" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="I14" t="s">
         <v>16</v>
       </c>
       <c r="J14" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="K14" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
       <c r="L14" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="M14" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="N14" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="O14" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="P14" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="Q14" t="s">
         <v>9</v>
       </c>
       <c r="R14" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="S14" t="s">
-        <v>295</v>
+        <v>287</v>
       </c>
       <c r="T14" t="s">
-        <v>312</v>
+        <v>304</v>
       </c>
       <c r="U14" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="V14" t="s">
-        <v>321</v>
+        <v>313</v>
       </c>
       <c r="W14" t="s">
-        <v>339</v>
+        <v>331</v>
       </c>
       <c r="X14" t="s">
-        <v>70</v>
+        <v>587</v>
       </c>
       <c r="Y14" t="s">
-        <v>355</v>
+        <v>347</v>
       </c>
       <c r="Z14" t="s">
-        <v>372</v>
+        <v>364</v>
       </c>
       <c r="AA14" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="AB14" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="AC14" t="s">
-        <v>405</v>
+        <v>397</v>
       </c>
       <c r="AD14" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="AE14" t="s">
-        <v>421</v>
+        <v>413</v>
       </c>
       <c r="AF14" t="s">
-        <v>438</v>
+        <v>430</v>
       </c>
       <c r="AG14" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="AH14" t="s">
-        <v>455</v>
+        <v>447</v>
       </c>
       <c r="AI14" t="s">
-        <v>471</v>
+        <v>463</v>
       </c>
       <c r="AJ14" t="s">
-        <v>488</v>
+        <v>480</v>
       </c>
       <c r="AK14" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="AL14" t="s">
-        <v>505</v>
+        <v>497</v>
       </c>
       <c r="AM14" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="AN14" t="s">
-        <v>522</v>
+        <v>514</v>
       </c>
       <c r="AO14" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="AP14" t="s">
-        <v>539</v>
+        <v>531</v>
       </c>
       <c r="AQ14" t="s">
-        <v>556</v>
+        <v>548</v>
       </c>
       <c r="AR14" t="s">
-        <v>556</v>
+        <v>548</v>
       </c>
       <c r="AS14" t="s">
         <v>37</v>
       </c>
       <c r="AT14" t="s">
-        <v>573</v>
+        <v>565</v>
       </c>
       <c r="AU14" t="s">
-        <v>590</v>
+        <v>582</v>
       </c>
     </row>
     <row r="15" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="B15" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C15" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="D15" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="E15" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="F15" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="G15" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="H15" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="I15" t="s">
         <v>16</v>
       </c>
       <c r="J15" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="K15" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
       <c r="L15" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="M15" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="N15" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="O15" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="P15" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="Q15" t="s">
         <v>2</v>
       </c>
       <c r="R15" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="S15" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="T15" t="s">
-        <v>313</v>
+        <v>305</v>
       </c>
       <c r="U15" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="V15" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="W15" t="s">
-        <v>340</v>
+        <v>332</v>
       </c>
       <c r="X15" t="s">
-        <v>55</v>
+        <v>29</v>
       </c>
       <c r="Y15" t="s">
-        <v>356</v>
+        <v>348</v>
       </c>
       <c r="Z15" t="s">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="AA15" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="AB15" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="AC15" t="s">
-        <v>406</v>
+        <v>398</v>
       </c>
       <c r="AD15" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="AE15" t="s">
-        <v>422</v>
+        <v>414</v>
       </c>
       <c r="AF15" t="s">
-        <v>439</v>
+        <v>431</v>
       </c>
       <c r="AG15" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="AH15" t="s">
-        <v>456</v>
+        <v>448</v>
       </c>
       <c r="AI15" t="s">
-        <v>472</v>
+        <v>464</v>
       </c>
       <c r="AJ15" t="s">
-        <v>489</v>
+        <v>481</v>
       </c>
       <c r="AK15" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="AL15" t="s">
-        <v>506</v>
+        <v>498</v>
       </c>
       <c r="AM15" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="AN15" t="s">
-        <v>523</v>
+        <v>515</v>
       </c>
       <c r="AO15" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="AP15" t="s">
-        <v>540</v>
+        <v>532</v>
       </c>
       <c r="AQ15" t="s">
-        <v>557</v>
+        <v>549</v>
       </c>
       <c r="AR15" t="s">
-        <v>557</v>
+        <v>549</v>
       </c>
       <c r="AS15" t="s">
         <v>7</v>
       </c>
       <c r="AT15" t="s">
-        <v>574</v>
+        <v>566</v>
       </c>
       <c r="AU15" t="s">
-        <v>591</v>
+        <v>583</v>
       </c>
     </row>
     <row r="16" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="B16" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C16" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="D16" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="E16" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="F16" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="G16" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="H16" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="I16" t="s">
         <v>44</v>
       </c>
       <c r="J16" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="K16" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="L16" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="M16" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="N16" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="O16" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="P16" t="s">
-        <v>281</v>
+        <v>273</v>
       </c>
       <c r="Q16" t="s">
         <v>2</v>
       </c>
       <c r="R16" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="S16" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="T16" t="s">
-        <v>314</v>
+        <v>306</v>
       </c>
       <c r="U16" t="s">
-        <v>78</v>
+        <v>3</v>
       </c>
       <c r="V16" t="s">
-        <v>323</v>
+        <v>315</v>
       </c>
       <c r="W16" t="s">
-        <v>341</v>
+        <v>333</v>
       </c>
       <c r="X16" t="s">
-        <v>79</v>
+        <v>586</v>
       </c>
       <c r="Y16" t="s">
-        <v>357</v>
+        <v>349</v>
       </c>
       <c r="Z16" t="s">
-        <v>374</v>
+        <v>366</v>
       </c>
       <c r="AA16" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="AB16" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="AC16" t="s">
-        <v>407</v>
+        <v>399</v>
       </c>
       <c r="AD16" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="AE16" t="s">
-        <v>423</v>
+        <v>415</v>
       </c>
       <c r="AF16" t="s">
-        <v>440</v>
+        <v>432</v>
       </c>
       <c r="AG16" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="AH16" t="s">
-        <v>457</v>
+        <v>449</v>
       </c>
       <c r="AI16" t="s">
-        <v>473</v>
+        <v>465</v>
       </c>
       <c r="AJ16" t="s">
-        <v>490</v>
+        <v>482</v>
       </c>
       <c r="AK16" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="AL16" t="s">
-        <v>507</v>
+        <v>499</v>
       </c>
       <c r="AM16" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="AN16" t="s">
-        <v>524</v>
+        <v>516</v>
       </c>
       <c r="AO16" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="AP16" t="s">
-        <v>541</v>
+        <v>533</v>
       </c>
       <c r="AQ16" t="s">
-        <v>558</v>
+        <v>550</v>
       </c>
       <c r="AR16" t="s">
-        <v>558</v>
+        <v>550</v>
       </c>
       <c r="AS16" t="s">
         <v>7</v>
       </c>
       <c r="AT16" t="s">
-        <v>575</v>
+        <v>567</v>
       </c>
       <c r="AU16" t="s">
-        <v>592</v>
+        <v>584</v>
       </c>
     </row>
     <row r="17" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="B17" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="C17" t="s">
+        <v>135</v>
+      </c>
+      <c r="D17" t="s">
+        <v>224</v>
+      </c>
+      <c r="E17" t="s">
+        <v>86</v>
+      </c>
+      <c r="F17" t="s">
+        <v>232</v>
+      </c>
+      <c r="G17" t="s">
         <v>143</v>
       </c>
-      <c r="D17" t="s">
-        <v>232</v>
-      </c>
-      <c r="E17" t="s">
-        <v>94</v>
-      </c>
-      <c r="F17" t="s">
-        <v>240</v>
-      </c>
-      <c r="G17" t="s">
-        <v>151</v>
-      </c>
       <c r="H17" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="I17" t="s">
         <v>44</v>
       </c>
       <c r="J17" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="K17" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="L17" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="M17" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="N17" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="O17" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="P17" t="s">
-        <v>281</v>
+        <v>273</v>
       </c>
       <c r="Q17" t="s">
         <v>9</v>
       </c>
       <c r="R17" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="S17" t="s">
-        <v>298</v>
+        <v>290</v>
       </c>
       <c r="T17" t="s">
-        <v>315</v>
+        <v>307</v>
       </c>
       <c r="U17" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="V17" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="W17" t="s">
-        <v>342</v>
+        <v>334</v>
       </c>
       <c r="X17" t="s">
         <v>40</v>
       </c>
       <c r="Y17" t="s">
-        <v>358</v>
+        <v>350</v>
       </c>
       <c r="Z17" t="s">
-        <v>375</v>
+        <v>367</v>
       </c>
       <c r="AA17" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="AB17" t="s">
-        <v>391</v>
+        <v>383</v>
       </c>
       <c r="AC17" t="s">
-        <v>408</v>
+        <v>400</v>
       </c>
       <c r="AD17" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="AE17" t="s">
-        <v>424</v>
+        <v>416</v>
       </c>
       <c r="AF17" t="s">
-        <v>441</v>
+        <v>433</v>
       </c>
       <c r="AG17" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="AH17" t="s">
-        <v>458</v>
+        <v>450</v>
       </c>
       <c r="AI17" t="s">
-        <v>474</v>
+        <v>466</v>
       </c>
       <c r="AJ17" t="s">
-        <v>491</v>
+        <v>483</v>
       </c>
       <c r="AK17" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="AL17" t="s">
-        <v>508</v>
+        <v>500</v>
       </c>
       <c r="AM17" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="AN17" t="s">
-        <v>525</v>
+        <v>517</v>
       </c>
       <c r="AO17" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="AP17" t="s">
-        <v>542</v>
+        <v>534</v>
       </c>
       <c r="AQ17" t="s">
-        <v>559</v>
+        <v>551</v>
       </c>
       <c r="AR17" t="s">
-        <v>559</v>
+        <v>551</v>
       </c>
       <c r="AS17" t="s">
         <v>14</v>
       </c>
       <c r="AT17" t="s">
-        <v>576</v>
+        <v>568</v>
       </c>
       <c r="AU17" t="s">
-        <v>593</v>
+        <v>585</v>
       </c>
     </row>
   </sheetData>

</xml_diff>